<commit_message>
added documentation on connectors used. To fit battery, iin battery sandwhich design as well as potential components on the back-side of the board
</commit_message>
<xml_diff>
--- a/BOM/Vital-Link-BOM2-V3.xlsx
+++ b/BOM/Vital-Link-BOM2-V3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Parry\Documents\GITHUB_desktop\Vital-link-hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BFAB6D-780B-4640-94D1-C09785756004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37AC4424-4758-447E-9653-863CEFE9B14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30816" yWindow="-96" windowWidth="30912" windowHeight="16752" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -477,6 +477,13 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -498,13 +505,6 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -725,47 +725,47 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="79.140625" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" customWidth="1"/>
-    <col min="4" max="4" width="96.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.3984375" customWidth="1"/>
+    <col min="2" max="2" width="79.1328125" customWidth="1"/>
+    <col min="3" max="3" width="34.59765625" customWidth="1"/>
+    <col min="4" max="4" width="96.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
         <v>2</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="31" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -779,8 +779,8 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="32"/>
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
@@ -791,8 +791,8 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="29"/>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="32"/>
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
@@ -803,8 +803,8 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="30"/>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="33"/>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
@@ -816,7 +816,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -831,7 +831,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -846,7 +846,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -857,7 +857,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A10" s="10" t="s">
         <v>12</v>
       </c>
@@ -886,7 +886,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="12">
         <v>1</v>
       </c>
@@ -916,7 +916,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="12">
         <v>2</v>
       </c>
@@ -946,7 +946,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="12">
         <v>3</v>
       </c>
@@ -976,7 +976,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="17.25" x14ac:dyDescent="0.45">
       <c r="A14" s="12">
         <v>4</v>
       </c>
@@ -989,22 +989,22 @@
       <c r="D14" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="39">
+      <c r="E14" s="28">
         <v>1</v>
       </c>
-      <c r="F14" s="40">
+      <c r="F14" s="29">
         <v>0</v>
       </c>
       <c r="G14" s="17">
         <v>8.59</v>
       </c>
-      <c r="H14" s="40">
+      <c r="H14" s="29">
         <f>(G14*E14)</f>
         <v>8.59</v>
       </c>
       <c r="I14" s="22"/>
     </row>
-    <row r="15" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="17.25" x14ac:dyDescent="0.45">
       <c r="A15" s="12">
         <v>5</v>
       </c>
@@ -1015,29 +1015,29 @@
       <c r="D15" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="39">
+      <c r="E15" s="28">
         <v>1</v>
       </c>
-      <c r="F15" s="40">
+      <c r="F15" s="29">
         <v>0</v>
       </c>
-      <c r="G15" s="40">
+      <c r="G15" s="29">
         <v>7.97</v>
       </c>
-      <c r="H15" s="40">
+      <c r="H15" s="29">
         <f>(G15*E15)</f>
         <v>7.97</v>
       </c>
       <c r="I15" s="22"/>
     </row>
-    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A16" s="12">
         <v>6</v>
       </c>
       <c r="B16" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="41" t="s">
+      <c r="C16" s="30" t="s">
         <v>41</v>
       </c>
       <c r="D16" s="25" t="s">
@@ -1052,13 +1052,13 @@
       <c r="G16" s="21">
         <v>6.83</v>
       </c>
-      <c r="H16" s="40">
+      <c r="H16" s="29">
         <f>(G16*E16)</f>
         <v>27.32</v>
       </c>
       <c r="I16" s="22"/>
     </row>
-    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="12"/>
       <c r="B19" s="7"/>
       <c r="C19" s="23"/>
@@ -1069,7 +1069,7 @@
       <c r="H19" s="16"/>
       <c r="I19" s="22"/>
     </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="12"/>
       <c r="B20" s="7"/>
       <c r="C20" s="23"/>
@@ -1080,7 +1080,7 @@
       <c r="H20" s="16"/>
       <c r="I20" s="22"/>
     </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A21" s="4"/>
       <c r="B21" s="24"/>
       <c r="C21" s="5"/>
@@ -1088,15 +1088,15 @@
       <c r="E21" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="31">
+      <c r="F21" s="34">
         <f>SUM(H11:H20)</f>
         <v>165.72399999999999</v>
       </c>
-      <c r="G21" s="32"/>
-      <c r="H21" s="33"/>
+      <c r="G21" s="35"/>
+      <c r="H21" s="36"/>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="4"/>
       <c r="B22" s="24"/>
       <c r="C22" s="5"/>
@@ -1104,15 +1104,15 @@
       <c r="E22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="34">
+      <c r="F22" s="37">
         <f>F21*0.12</f>
         <v>19.886879999999998</v>
       </c>
-      <c r="G22" s="35"/>
-      <c r="H22" s="36"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="39"/>
       <c r="I22" s="4"/>
     </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A23" s="4"/>
       <c r="B23" s="24"/>
       <c r="C23" s="5"/>
@@ -1120,15 +1120,15 @@
       <c r="E23" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F23" s="37">
+      <c r="F23" s="40">
         <f>SUM(F21:H22)</f>
         <v>185.61087999999998</v>
       </c>
-      <c r="G23" s="35"/>
-      <c r="H23" s="36"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="39"/>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="4"/>
       <c r="B24" s="24"/>
       <c r="C24" s="5"/>
@@ -1139,19 +1139,19 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="24"/>
     </row>
-    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="24"/>
     </row>
-    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="24"/>
     </row>
-    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="24"/>
     </row>
-    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="24"/>
     </row>
   </sheetData>

</xml_diff>